<commit_message>
feat: Melhorias M5 a M7
</commit_message>
<xml_diff>
--- a/docs/avaliacao/plano_de_acao_melhorias.xlsx
+++ b/docs/avaliacao/plano_de_acao_melhorias.xlsx
@@ -912,7 +912,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Não iniciada</t>
+          <t>Em andamento: detector e regeneração implementados (43 testes unitários ok); falta reexecutar com qwen2.5:7b</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -968,7 +968,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Não iniciada</t>
+          <t>Em andamento: 12 cenários (32 turnos) e modo conversa no executor prontos; falta executar com qwen2.5:7b</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Não iniciada</t>
+          <t>Em andamento: filtro por nota do LLM (0–2) e mensagem de ausência de evidência implementados (65 testes ok); falta medir com qwen2.5:7b</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
     </row>
@@ -1921,7 +1921,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
     </row>
@@ -1981,7 +1981,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
     </row>
@@ -2011,7 +2011,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
     </row>
@@ -2071,7 +2071,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
     </row>

</xml_diff>